<commit_message>
Remove (X) markers from phone numbers in 문자발송 리스트
카톡 친구추가 불가 표시용 '(X)' 마커 80건을 전화번호에서 제거해 깨끗한 번호로 정리.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EjGkfThxVyyC2xq8RJdcuC
</commit_message>
<xml_diff>
--- a/체험단_문자발송_리스트.xlsx
+++ b/체험단_문자발송_리스트.xlsx
@@ -5524,7 +5524,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>010-7490-3175(X)</t>
+          <t>010-7490-3175</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>010-7360-5998(X)</t>
+          <t>010-7360-5998</t>
         </is>
       </c>
     </row>
@@ -5548,7 +5548,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>010-2187-1826(X)</t>
+          <t>010-2187-1826</t>
         </is>
       </c>
     </row>
@@ -5560,7 +5560,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>010-2830-5915(X)</t>
+          <t>010-2830-5915</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>010-6699-8867(X)</t>
+          <t>010-6699-8867</t>
         </is>
       </c>
     </row>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>010-2189-6146(X)</t>
+          <t>010-2189-6146</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>010-8039-0914(X)</t>
+          <t>010-8039-0914</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>010-8053-0716(X)</t>
+          <t>010-8053-0716</t>
         </is>
       </c>
     </row>
@@ -5620,7 +5620,7 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>010-4044-9770(X)</t>
+          <t>010-4044-9770</t>
         </is>
       </c>
     </row>
@@ -5632,7 +5632,7 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>010-5722-2606(X)</t>
+          <t>010-5722-2606</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>010-2475-5632(X)</t>
+          <t>010-2475-5632</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>010-3953-3976(X)</t>
+          <t>010-3953-3976</t>
         </is>
       </c>
     </row>
@@ -5668,7 +5668,7 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>010-4985-0227(X)</t>
+          <t>010-4985-0227</t>
         </is>
       </c>
     </row>
@@ -5680,7 +5680,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>010-4080-0816(X)</t>
+          <t>010-4080-0816</t>
         </is>
       </c>
     </row>
@@ -5692,7 +5692,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>010-6829-1853(X)</t>
+          <t>010-6829-1853</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>010-2459-5439(X)</t>
+          <t>010-2459-5439</t>
         </is>
       </c>
     </row>
@@ -5716,7 +5716,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>010-8832-8321(X)</t>
+          <t>010-8832-8321</t>
         </is>
       </c>
     </row>
@@ -5728,7 +5728,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>010-4285-4808(X)</t>
+          <t>010-4285-4808</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>010-2184-2406(X)</t>
+          <t>010-2184-2406</t>
         </is>
       </c>
     </row>
@@ -5752,7 +5752,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>010-5267-9954(X)</t>
+          <t>010-5267-9954</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>010-2190-6977(X)</t>
+          <t>010-2190-6977</t>
         </is>
       </c>
     </row>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>010-7479-7379(X)</t>
+          <t>010-7479-7379</t>
         </is>
       </c>
     </row>
@@ -5788,7 +5788,7 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>010-9748-6355(X)</t>
+          <t>010-9748-6355</t>
         </is>
       </c>
     </row>
@@ -5800,7 +5800,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>010-6470-3314(X)</t>
+          <t>010-6470-3314</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>010-4259-7925(X)</t>
+          <t>010-4259-7925</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5824,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>010-7297-2589(X)</t>
+          <t>010-7297-2589</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>010-5756-2674(X)</t>
+          <t>010-5756-2674</t>
         </is>
       </c>
     </row>
@@ -5848,7 +5848,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>010-8363-6572(X)</t>
+          <t>010-8363-6572</t>
         </is>
       </c>
     </row>
@@ -5860,7 +5860,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>010-4345-9923(X)</t>
+          <t>010-4345-9923</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>010-2007-3348(X)</t>
+          <t>010-2007-3348</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5884,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>010-2832-8564(X)</t>
+          <t>010-2832-8564</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5896,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>010-6829-3373(X)</t>
+          <t>010-6829-3373</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5908,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>010-2267-4804(X)</t>
+          <t>010-2267-4804</t>
         </is>
       </c>
     </row>
@@ -5920,7 +5920,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>010-5450-0322(X)</t>
+          <t>010-5450-0322</t>
         </is>
       </c>
     </row>
@@ -5932,7 +5932,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>010-5967-6921(X)</t>
+          <t>010-5967-6921</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>010-8249-5345(X)</t>
+          <t>010-8249-5345</t>
         </is>
       </c>
     </row>
@@ -5956,7 +5956,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>010-4291-7733(X)</t>
+          <t>010-4291-7733</t>
         </is>
       </c>
     </row>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>010-7307-2721(X)</t>
+          <t>010-7307-2721</t>
         </is>
       </c>
     </row>
@@ -5980,7 +5980,7 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>010-6862-0278(X)</t>
+          <t>010-6862-0278</t>
         </is>
       </c>
     </row>
@@ -5992,7 +5992,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>010-5865-4517(X)</t>
+          <t>010-5865-4517</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6004,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>010-2895-5280(X)</t>
+          <t>010-2895-5280</t>
         </is>
       </c>
     </row>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>010-8062-6302(X)</t>
+          <t>010-8062-6302</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6028,7 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>010-3929-1572(X)</t>
+          <t>010-3929-1572</t>
         </is>
       </c>
     </row>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>010-9778-4323(X)</t>
+          <t>010-9778-4323</t>
         </is>
       </c>
     </row>
@@ -6052,7 +6052,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>010-5023-3663(X)</t>
+          <t>010-5023-3663</t>
         </is>
       </c>
     </row>
@@ -6064,7 +6064,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>010-6842-4425(X)</t>
+          <t>010-6842-4425</t>
         </is>
       </c>
     </row>
@@ -6076,7 +6076,7 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>010-6624-9810(X)</t>
+          <t>010-6624-9810</t>
         </is>
       </c>
     </row>
@@ -6088,7 +6088,7 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>010-5562-2801(X)</t>
+          <t>010-5562-2801</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>010-8022-1556(X)</t>
+          <t>010-8022-1556</t>
         </is>
       </c>
     </row>
@@ -6112,7 +6112,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>010-5400-5103(X)</t>
+          <t>010-5400-5103</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>010-8226-4156(X)</t>
+          <t>010-8226-4156</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6136,7 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>010-6827-1963(X)</t>
+          <t>010-6827-1963</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>010-7623-4157(X)</t>
+          <t>010-7623-4157</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>010-4452-3616(X)</t>
+          <t>010-4452-3616</t>
         </is>
       </c>
     </row>
@@ -6172,7 +6172,7 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>010-6740-2311(X)</t>
+          <t>010-6740-2311</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>010-9887-2617(X)</t>
+          <t>010-9887-2617</t>
         </is>
       </c>
     </row>
@@ -6196,7 +6196,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>010-4830-7629(X)</t>
+          <t>010-4830-7629</t>
         </is>
       </c>
     </row>
@@ -6208,7 +6208,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>010-9726-1156(X)</t>
+          <t>010-9726-1156</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>010-9642-7704(X)</t>
+          <t>010-9642-7704</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6232,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>010-7444-6546(X)</t>
+          <t>010-7444-6546</t>
         </is>
       </c>
     </row>
@@ -6244,7 +6244,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>010-8925-5060(X)</t>
+          <t>010-8925-5060</t>
         </is>
       </c>
     </row>
@@ -6256,31 +6256,31 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>010-8306-1277(X)</t>
+          <t>010-8306-1277</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>010-8991-7784(X)</t>
+          <t>010-8991-7784</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>010-8991-7784(X)</t>
+          <t>010-8991-7784</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>010-239-6219(X)</t>
+          <t>010-239-6219</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>010-239-6219(X)</t>
+          <t>010-239-6219</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>010-2942-7290(X)</t>
+          <t>010-2942-7290</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6304,7 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>010-6895-8965(X)</t>
+          <t>010-6895-8965</t>
         </is>
       </c>
     </row>
@@ -6316,7 +6316,7 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>010-9538-3220(X)</t>
+          <t>010-9538-3220</t>
         </is>
       </c>
     </row>
@@ -6328,7 +6328,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>010-2297-7675(X)</t>
+          <t>010-2297-7675</t>
         </is>
       </c>
     </row>
@@ -6340,7 +6340,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>010-2150-0069(X)</t>
+          <t>010-2150-0069</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>010-6715-5322(X)</t>
+          <t>010-6715-5322</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>010-8096-5458(X)</t>
+          <t>010-8096-5458</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>010-6554-4261(X)</t>
+          <t>010-6554-4261</t>
         </is>
       </c>
     </row>
@@ -6388,7 +6388,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>010-6827-9560(X)</t>
+          <t>010-6827-9560</t>
         </is>
       </c>
     </row>
@@ -6400,7 +6400,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>010-8210-8885(X)</t>
+          <t>010-8210-8885</t>
         </is>
       </c>
     </row>
@@ -6412,7 +6412,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>010-4413-0372(X)</t>
+          <t>010-4413-0372</t>
         </is>
       </c>
     </row>
@@ -6424,7 +6424,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>010-5727-7518(X)</t>
+          <t>010-5727-7518</t>
         </is>
       </c>
     </row>

</xml_diff>